<commit_message>
Small changes in names
</commit_message>
<xml_diff>
--- a/Courses_Data.xlsx
+++ b/Courses_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/antonipieszczoch/Desktop/Optimised Math Learning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6065C5D3-7D5D-2F4D-9870-B168B9BDAAAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9F4C6614-F7D1-0143-8377-BB391264A977}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="16000" xr2:uid="{403890A9-C917-BC41-96EF-6BB1034E316E}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="16000" xr2:uid="{F53E98A7-EF1E-924B-8C9E-487A44BE2458}"/>
   </bookViews>
   <sheets>
     <sheet name="Courses_Data" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="47">
   <si>
     <t>Macro_Topic</t>
   </si>
@@ -46,31 +46,40 @@
     <t>Function_Name</t>
   </si>
   <si>
+    <t>Trap_Message</t>
+  </si>
+  <si>
+    <t>Wrong_Message</t>
+  </si>
+  <si>
     <t>Fractions</t>
   </si>
   <si>
-    <t>Addition and Substraction</t>
+    <t>Addition</t>
   </si>
   <si>
     <t>Identical Denominators</t>
   </si>
   <si>
-    <t>Denominators must match. Numerators 1-9. Sum must be less than denominator. Constraint: Final sum must not be simplifiable (e.g., avoid 2/4 or 4/4). Output the raw fraction.</t>
+    <t>Denominators must match. Numerators 1-9. Sum must be less than denominator. Constraint: Final sum must not be simplifiable.</t>
   </si>
   <si>
     <t>Calculate by adding numerator A to numerator B, AND adding denominator A to denominator B. Format as a/b.</t>
   </si>
   <si>
-    <t>Calculate by making a +/- 1 arithmetic error in the correct numerator sum. Keep the denominator correct.</t>
+    <t>Calculate by making a +/- 1 arithmetic error in the correct numerator sum.</t>
   </si>
   <si>
     <t>add_fractions_simple</t>
   </si>
   <si>
+    <t>Niezupełnie. To jest zwykły błąd obliczeniowy w liczniku. Spróbuj jeszcze raz!</t>
+  </si>
+  <si>
     <t>Single Conversion</t>
   </si>
   <si>
-    <t>Denominators differ. One is a direct multiple of the other (e.g., 2 &amp; 4). Constraint:Final sum must not be simplifiable.</t>
+    <t>Denominators differ. One is a direct multiple of the other.</t>
   </si>
   <si>
     <t>Calculate by adding the unscaled numerator of fraction A to the numerator of fraction B, placing the sum over the larger denominator.</t>
@@ -82,13 +91,19 @@
     <t>add_fractions_single_conversion</t>
   </si>
   <si>
+    <t>Dodałeś liczniki bez uprzedniego rozszerzenia ułamka!</t>
+  </si>
+  <si>
+    <t>Pomnożyłeś liczniki zamiast je dodać!</t>
+  </si>
+  <si>
     <t>Double Conversion</t>
   </si>
   <si>
-    <t>Denominators are coprime (e.g., 3 &amp; 4). Requires mutual multiplication. Constraint: Final sum must not be simplifiable.</t>
-  </si>
-  <si>
-    <t>Calculate by adding numerator to numerator and multiplying the denominators directly.</t>
+    <t>Denominators are coprime. Requires mutual multiplication.</t>
+  </si>
+  <si>
+    <t>Calculate by adding numerator to numerator and denominator to denominator directly.</t>
   </si>
   <si>
     <t>Calculate using the correct common denominator, but fail to multiply the numerators by their respective scaling factors.</t>
@@ -97,10 +112,16 @@
     <t>add_fractions_complex</t>
   </si>
   <si>
+    <t>Błąd! Dodałeś do siebie liczniki i mianowniki.</t>
+  </si>
+  <si>
+    <t>Znalazłeś wspólny mianownik, ale zapomniałeś rozszerzyć liczniki!</t>
+  </si>
+  <si>
     <t>Mixed Numbers (Easy)</t>
   </si>
   <si>
-    <t>Whole numbers included. Denominators are identical or require Single Conversion. Constraint: The fractional sum must not exceed 1.</t>
+    <t>Whole numbers included. Identical Denominators.</t>
   </si>
   <si>
     <t>Calculate by adding the whole numbers correctly, but applying the Level 1 trap (adding denominators) to the fractional part.</t>
@@ -112,19 +133,34 @@
     <t>add_mixed_numbers_simple</t>
   </si>
   <si>
+    <t>Całości dodane świetnie, ale mianowniki ułamków również zostały dodane. Mianownik musi zostać bez zmian!</t>
+  </si>
+  <si>
+    <t>Pojawił się błąd obliczeniowy podczas dodawania liczników.</t>
+  </si>
+  <si>
     <t>The Final Boss</t>
   </si>
   <si>
-    <t>Mixed numbers. Denominators are coprime. Constraint: Sum of the fractions must exceed 1 (requires carrying over to the whole number).</t>
-  </si>
-  <si>
-    <t>Calculate by leaving the fractional part as an improper fraction and failing to carry the 1 over to the whole number sum.</t>
+    <t>Mixed numbers. Denominators are coprime.</t>
   </si>
   <si>
     <t>Calculate by finding the common denominator, but adding the original unscaled numerators together.</t>
   </si>
   <si>
+    <t>Calculate by adding the whole numbers, adding the numerators, and adding the denominators.</t>
+  </si>
+  <si>
     <t>add_mixed_numbers_complex</t>
+  </si>
+  <si>
+    <t>Zapomniałeś rozszerzyć liczniki przed dodaniem ułamków!</t>
+  </si>
+  <si>
+    <t>Błąd! Dodałeś do siebie mianowniki.</t>
+  </si>
+  <si>
+    <t>Dodałeś mianowniki. W dodawaniu ułamków mianownik zostaje bez zmian.</t>
   </si>
 </sst>
 </file>
@@ -984,11 +1020,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{081EDEFC-3A96-B142-AFD4-AFCA554E65C7}">
-  <dimension ref="A1:H6"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4696064F-12C5-9F40-B02D-0B74D749CBBB}">
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1013,135 +1049,171 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
+        <v>46</v>
+      </c>
+      <c r="J2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s">
+      <c r="B3" t="s">
         <v>11</v>
-      </c>
-      <c r="F2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>9</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E3" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="G3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H3" t="s">
-        <v>19</v>
+        <v>22</v>
+      </c>
+      <c r="I3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J3" t="s">
+        <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C4">
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F4" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G4" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="H4" t="s">
-        <v>24</v>
+        <v>29</v>
+      </c>
+      <c r="I4" t="s">
+        <v>30</v>
+      </c>
+      <c r="J4" t="s">
+        <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C5">
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="E5" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="F5" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="G5" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="H5" t="s">
-        <v>29</v>
+        <v>36</v>
+      </c>
+      <c r="I5" t="s">
+        <v>37</v>
+      </c>
+      <c r="J5" t="s">
+        <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C6">
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="E6" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="F6" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="G6" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="H6" t="s">
-        <v>34</v>
+        <v>43</v>
+      </c>
+      <c r="I6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J6" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>